<commit_message>
feat: implement complete quest system with progress tracking and completion #348
- Add quest system with progress tracking and completion logic
- Implement quest database schema and data models
- Add quest builtin functions for Lua scripting
- Create quest protocol handlers for client communication
- Update character system to support quest management
- Add quest-related mob scripts and interactions
- Implement HTTP API endpoints for quest management
- Update FlatBuffer protocol definitions for quest system
- Add quest and reward data tables
</commit_message>
<xml_diff>
--- a/resources/table/quest.xlsx
+++ b/resources/table/quest.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\fb\resources\table\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB09A176-241F-4304-92BC-02C7BA615A9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFDECA53-EB97-47C0-8973-DE5515B18967}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-135" windowWidth="38640" windowHeight="21120" xr2:uid="{D06B357D-EBE0-49AC-A207-4E89A5AA0593}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{D06B357D-EBE0-49AC-A207-4E89A5AA0593}"/>
   </bookViews>
   <sheets>
     <sheet name="quest" sheetId="1" r:id="rId1"/>
@@ -154,7 +154,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -170,7 +170,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 테마">
   <a:themeElements>
     <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
@@ -469,7 +469,9 @@
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="4" width="9" style="1"/>
+    <col min="1" max="1" width="9" style="1"/>
+    <col min="2" max="2" width="8.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="9" style="1"/>
     <col min="5" max="5" width="11.375" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="16384" width="9" style="1"/>
   </cols>

</xml_diff>

<commit_message>
feat: add exp DSL type and improve quest system #351
- Add exp DSL type for experience rewards
- Update quest progress and step increment logic
- Add remove_quest command for quest management
- Improve quest parameter handling in scripts
- Update quest and reward data tables
</commit_message>
<xml_diff>
--- a/resources/table/quest.xlsx
+++ b/resources/table/quest.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFDECA53-EB97-47C0-8973-DE5515B18967}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{841A55A7-D9F7-4813-9018-C28E9C0413AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{D06B357D-EBE0-49AC-A207-4E89A5AA0593}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="15">
   <si>
     <t>id</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -79,6 +79,10 @@
   </si>
   <si>
     <t>*uint32</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>level(10)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -531,6 +535,9 @@
       <c r="A4" s="1">
         <v>1</v>
       </c>
+      <c r="B4" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="C4" s="1" t="s">
         <v>7</v>
       </c>

</xml_diff>